<commit_message>
feat: data 配下の TSV 群と styles.json を出力する
Book.load で sheets.json に加え、value/type/formula/format/formatted_value/merge/style の各 TSV を書き出す。formatted_value は styles を参照した簡易表示、失敗時は value にフォールバック。merge はドキュメント規約の 0,0 / 0,1 / -1,-1。style は cellXf インデックス ID のみ。styles.json には ID ごとの numFmtId・formatCode・restore_xml（xf 断片）をまとめる。tmp を .gitignore に追加。

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/input/sampledata.xlsx
+++ b/src/test/resources/input/sampledata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okuyama/Documents/projects/excel002/src/test/resources/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F994A0-7627-D542-BDCA-180C3A5EAA67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC364169-7657-C94B-99A4-CBB95491AB19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="91980" yWindow="28060" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="76800" yWindow="22100" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="10">
   <si>
     <t>sampledata</t>
   </si>
@@ -1177,4 +1178,30 @@
   <phoneticPr fontId="18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1452489A-43CF-7C47-8329-D76A122C3DFD}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="18"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>